<commit_message>
Loveless bib removed from Gen 33
</commit_message>
<xml_diff>
--- a/data/post2002DB-v3.xlsx
+++ b/data/post2002DB-v3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hildad/Documents/GitHub/lyingpendatabases/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hildad/Github/lyingpendatabases/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5510202-D7C3-DA4A-A52C-88E09EB40E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47049A9-0CEB-0D47-AF97-A08F8E032FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{CB7DAB00-11D3-3A4F-BDDA-5DEC01C2CC59}"/>
   </bookViews>
@@ -5393,98 +5393,6 @@
   </si>
   <si>
     <r>
-      <t>Eshel, Esther and Hanan Eshel. 2005. “New Fragments from Qumran: 4QGen</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>&lt;sup&gt;f&lt;/sup&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>, 4QIsa</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>&lt;sup&gt;b&lt;/sup&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>, 4Q226, 8QGen, and XQpapEnoch.” &lt;i&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>DSD</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>&lt;/i&gt; 12: 134–57, see 135–37.
-Loveless, Gary and Stephanie. 2012. &lt;i&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>Dead Sea Scrolls and The Bible: Ancient Artifacts, Timeless Treasures</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>&lt;/i&gt;. Forth Worth: Southwestern Baptist Theological Seminary. See pp. 100–1.
-Tigchelaar, Eibert. 2012. “Notes on the Three Qumran-Type Yadin Fragments Leading to a Discussion of Identification, Attribution, Provenance, and Names.” &lt;i&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>DSD</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aleo Light"/>
-      </rPr>
-      <t>&lt;/i&gt; 19: 198–214, see pp. 212–13.</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>Identified (and sold?) as 4Q33 (4QDeut</t>
     </r>
     <r>
@@ -6678,6 +6586,80 @@
 (William Kando) [Fields 2011]
 2011– : $35–70 million (William Kando)
 2013: upwards of £26 million (Lee Biondi according to Parker 2013)</t>
+  </si>
+  <si>
+    <r>
+      <t>Eshel, Esther and Hanan Eshel. 2005. “New Fragments from Qumran: 4QGen</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aleo Light"/>
+      </rPr>
+      <t>&lt;sup&gt;f&lt;/sup&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aleo Light"/>
+      </rPr>
+      <t>, 4QIsa</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aleo Light"/>
+      </rPr>
+      <t>&lt;sup&gt;b&lt;/sup&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aleo Light"/>
+      </rPr>
+      <t>, 4Q226, 8QGen, and XQpapEnoch.” &lt;i&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aleo Light"/>
+      </rPr>
+      <t>DSD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aleo Light"/>
+      </rPr>
+      <t>&lt;/i&gt; 12: 134–57, see 135–37.
+Tigchelaar, Eibert. 2012. “Notes on the Three Qumran-Type Yadin Fragments Leading to a Discussion of Identification, Attribution, Provenance, and Names.” &lt;i&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aleo Light"/>
+      </rPr>
+      <t>DSD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aleo Light"/>
+      </rPr>
+      <t>&lt;/i&gt; 19: 198–214, see pp. 212–13.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -6986,23 +6968,6 @@
         <patternFill patternType="solid"/>
       </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <sz val="10"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
@@ -7731,6 +7696,23 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -7771,50 +7753,44 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4CEA2365-8B2D-5143-803D-6D4FB4E86B2D}" name="Post_2002_Fragments" displayName="Post_2002_Fragments" ref="A1:U104" totalsRowShown="0" headerRowDxfId="22" dataDxfId="0">
-  <autoFilter ref="A1:U104" xr:uid="{714D2FCE-A08D-C943-80D3-6D216A6BD6AA}">
-    <filterColumn colId="13">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4CEA2365-8B2D-5143-803D-6D4FB4E86B2D}" name="Post_2002_Fragments" displayName="Post_2002_Fragments" ref="A1:U104" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="A1:U104" xr:uid="{714D2FCE-A08D-C943-80D3-6D216A6BD6AA}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U104">
     <sortCondition ref="A1:A104"/>
   </sortState>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{4EFD41BC-5BFD-4E46-A5F1-7E906C6102C5}" name="Item No." dataDxfId="21"/>
-    <tableColumn id="11" xr3:uid="{AE8ADACF-00B6-7649-B9A0-10958EB147C4}" name="Item Name" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{4EFD41BC-5BFD-4E46-A5F1-7E906C6102C5}" name="Item No." dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{AE8ADACF-00B6-7649-B9A0-10958EB147C4}" name="Item Name" dataDxfId="19">
       <calculatedColumnFormula>IF(ISNUMBER(Post_2002_Fragments[[#This Row],[Item No.]]),_xlfn.CONCAT(IF(Post_2002_Fragments[[#This Row],[DSS F. No.]]="",IF(ISNUMBER(SEARCH("Unidentified",Post_2002_Fragments[[#This Row],[Content]])),"Unidentified",Post_2002_Fragments[[#This Row],[Content]]),_xlfn.CONCAT("DSS F.",Post_2002_Fragments[[#This Row],[DSS F. No.]]," ",Post_2002_Fragments[[#This Row],[DSS F. Name]]))),Post_2002_Fragments[[#This Row],[Item No.]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{4DDC7D22-B286-AD43-9DF0-FC7A4BACEAA9}" name="DSS F. No." dataDxfId="19"/>
-    <tableColumn id="14" xr3:uid="{46E1AC7F-0FC2-3041-B3E2-F0809B37FB08}" name="DSS F. Name" dataDxfId="18"/>
-    <tableColumn id="15" xr3:uid="{F93B8E3F-E2A9-9C46-8798-E2857A037AA3}" name="Content" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{11BD8FB7-E8BA-EE49-B0FE-64041D98EB57}" name="Incorrect DSS Identifications" dataDxfId="16"/>
-    <tableColumn id="32" xr3:uid="{9E02593A-E84E-124C-84CB-F3EC28D64481}" name="Recently Invented DSS Manuscript Labels" dataDxfId="15"/>
-    <tableColumn id="28" xr3:uid="{7CFA9B31-34B3-1249-944A-FE370EC2B25E}" name="Siglum (Name) in Tov, Revised Lists (2010)" dataDxfId="14"/>
-    <tableColumn id="29" xr3:uid="{F6F3730C-3E78-9640-BD99-2AABB1F5151F}" name="Siglum and Fragment Number in Accordance" dataDxfId="13"/>
-    <tableColumn id="19" xr3:uid="{F6AC96E7-4BB0-A14A-9245-5E3480975FD9}" name="Current Owner" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{142CBA6D-F3C5-874F-9A10-B4D0D370D4AD}" name="Collection No." dataDxfId="11"/>
-    <tableColumn id="35" xr3:uid="{C459176B-7CFF-7741-81F6-696F6DDA7AC2}" name="Alleged Provenance" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{E85C9271-D71B-2347-AC6C-CB969F40EC18}" name="Sale (➤), Donation (➢), and Collaboration (→)" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{B3E9F172-B29F-F14F-9417-580D64DFAF47}" name="Asking Price" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{91E1017E-7A63-B64C-B629-BFE8CFEC540C}" name="Purchase Price_x000a_Dealer/Seller ➤ Collector/Buyer" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{652C307D-EFC9-A44D-B6B7-7E5415A0E08F}" name="Lines" dataDxfId="6"/>
-    <tableColumn id="16" xr3:uid="{0B1022CB-F629-D54B-ACE5-24014EED6254}" name="Measurements_x000a_(in cm)" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{4665D607-2EED-974F-8F27-60FF09978FC3}" name="Principal Edition" dataDxfId="4"/>
-    <tableColumn id="34" xr3:uid="{516E9851-23BA-4E51-9FAE-45E15B80C08C}" name="Bibliography" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{BA6B59E9-7DD8-3F41-B53D-D836BA825549}" name="Composition" dataDxfId="2"/>
-    <tableColumn id="17" xr3:uid="{9B268625-BF17-7245-969F-CCAF877DBC86}" name="Canonical Categorisation" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{4DDC7D22-B286-AD43-9DF0-FC7A4BACEAA9}" name="DSS F. No." dataDxfId="18"/>
+    <tableColumn id="14" xr3:uid="{46E1AC7F-0FC2-3041-B3E2-F0809B37FB08}" name="DSS F. Name" dataDxfId="17"/>
+    <tableColumn id="15" xr3:uid="{F93B8E3F-E2A9-9C46-8798-E2857A037AA3}" name="Content" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{11BD8FB7-E8BA-EE49-B0FE-64041D98EB57}" name="Incorrect DSS Identifications" dataDxfId="15"/>
+    <tableColumn id="32" xr3:uid="{9E02593A-E84E-124C-84CB-F3EC28D64481}" name="Recently Invented DSS Manuscript Labels" dataDxfId="14"/>
+    <tableColumn id="28" xr3:uid="{7CFA9B31-34B3-1249-944A-FE370EC2B25E}" name="Siglum (Name) in Tov, Revised Lists (2010)" dataDxfId="13"/>
+    <tableColumn id="29" xr3:uid="{F6F3730C-3E78-9640-BD99-2AABB1F5151F}" name="Siglum and Fragment Number in Accordance" dataDxfId="12"/>
+    <tableColumn id="19" xr3:uid="{F6AC96E7-4BB0-A14A-9245-5E3480975FD9}" name="Current Owner" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{142CBA6D-F3C5-874F-9A10-B4D0D370D4AD}" name="Collection No." dataDxfId="10"/>
+    <tableColumn id="35" xr3:uid="{C459176B-7CFF-7741-81F6-696F6DDA7AC2}" name="Alleged Provenance" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{E85C9271-D71B-2347-AC6C-CB969F40EC18}" name="Sale (➤), Donation (➢), and Collaboration (→)" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{B3E9F172-B29F-F14F-9417-580D64DFAF47}" name="Asking Price" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{91E1017E-7A63-B64C-B629-BFE8CFEC540C}" name="Purchase Price_x000a_Dealer/Seller ➤ Collector/Buyer" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{652C307D-EFC9-A44D-B6B7-7E5415A0E08F}" name="Lines" dataDxfId="5"/>
+    <tableColumn id="16" xr3:uid="{0B1022CB-F629-D54B-ACE5-24014EED6254}" name="Measurements_x000a_(in cm)" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{4665D607-2EED-974F-8F27-60FF09978FC3}" name="Principal Edition" dataDxfId="3"/>
+    <tableColumn id="34" xr3:uid="{516E9851-23BA-4E51-9FAE-45E15B80C08C}" name="Bibliography" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{BA6B59E9-7DD8-3F41-B53D-D836BA825549}" name="Composition" dataDxfId="1"/>
+    <tableColumn id="17" xr3:uid="{9B268625-BF17-7245-969F-CCAF877DBC86}" name="Canonical Categorisation" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -7852,7 +7828,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -7958,7 +7934,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8100,7 +8076,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -8212,10 +8188,10 @@
   <sheetData>
     <row r="1" spans="1:21" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>0</v>
@@ -8227,19 +8203,19 @@
         <v>2</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>545</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>546</v>
-      </c>
       <c r="H1" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>491</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>492</v>
-      </c>
       <c r="J1" s="3" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>3</v>
@@ -8248,10 +8224,10 @@
         <v>4</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="O1" s="3" t="s">
         <v>5</v>
@@ -8260,22 +8236,22 @@
         <v>6</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="T1" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="U1" s="3" t="s">
         <v>556</v>
       </c>
-      <c r="U1" s="3" t="s">
-        <v>557</v>
-      </c>
     </row>
-    <row r="2" spans="1:21" ht="92" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:21" ht="92" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -8304,7 +8280,7 @@
         <v>8</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="N2" s="9"/>
       <c r="O2" s="9"/>
@@ -8315,16 +8291,16 @@
         <v>13</v>
       </c>
       <c r="R2" s="5" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="S2" s="14" t="s">
         <v>14</v>
       </c>
       <c r="T2" s="20" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="U2" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="193" x14ac:dyDescent="0.2">
@@ -8341,7 +8317,7 @@
         <v>15</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>16</v>
@@ -8358,13 +8334,13 @@
         <v>17</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="P3" s="9" t="s">
         <v>20</v>
@@ -8373,19 +8349,19 @@
         <v>21</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="S3" s="14" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="T3" s="20" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="U3" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="130" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:21" ht="130" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -8407,7 +8383,7 @@
       <c r="H4" s="5"/>
       <c r="I4" s="9"/>
       <c r="J4" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>24</v>
@@ -8416,7 +8392,7 @@
         <v>458</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="N4" s="9"/>
       <c r="O4" s="9"/>
@@ -8433,13 +8409,13 @@
         <v>27</v>
       </c>
       <c r="T4" s="20" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="U4" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="146" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:21" ht="73" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -8477,19 +8453,19 @@
         <v>33</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="S5" s="16" t="s">
-        <v>459</v>
+        <v>594</v>
       </c>
       <c r="T5" s="20" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="U5" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="356" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:21" ht="370" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -8504,7 +8480,7 @@
         <v>34</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="5" t="s">
@@ -8513,7 +8489,7 @@
       <c r="H6" s="5"/>
       <c r="I6" s="9"/>
       <c r="J6" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>35</v>
@@ -8539,13 +8515,13 @@
         <v>42</v>
       </c>
       <c r="T6" s="20" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="U6" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="409.6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:21" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -8563,13 +8539,13 @@
         <v>44</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="15"/>
       <c r="I7" s="11"/>
       <c r="J7" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>45</v>
@@ -8595,10 +8571,10 @@
         <v>52</v>
       </c>
       <c r="T7" s="20" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="U7" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="8" spans="1:21" ht="195" x14ac:dyDescent="0.2">
@@ -8629,7 +8605,7 @@
       </c>
       <c r="M8" s="9"/>
       <c r="N8" s="9" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="O8" s="9"/>
       <c r="P8" s="9" t="s">
@@ -8643,13 +8619,13 @@
         <v>58</v>
       </c>
       <c r="T8" s="20" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="U8" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -8681,13 +8657,13 @@
         <v>60</v>
       </c>
       <c r="T9" s="20" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="U9" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="99.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:21" ht="99.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -8715,7 +8691,7 @@
         <v>67</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K10" s="5" t="s">
         <v>63</v>
@@ -8739,13 +8715,13 @@
         <v>69</v>
       </c>
       <c r="T10" s="20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U10" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="156.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:21" ht="156.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -8763,7 +8739,7 @@
         <v>71</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="5" t="s">
@@ -8773,7 +8749,7 @@
         <v>74</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>72</v>
@@ -8797,13 +8773,13 @@
         <v>77</v>
       </c>
       <c r="T11" s="20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U11" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -8835,13 +8811,13 @@
         <v>60</v>
       </c>
       <c r="T12" s="20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U12" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="110" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:21" ht="75" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -8864,7 +8840,7 @@
         <v>80</v>
       </c>
       <c r="M13" s="9" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="N13" s="9"/>
       <c r="O13" s="9"/>
@@ -8877,13 +8853,13 @@
         <v>81</v>
       </c>
       <c r="T13" s="20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U13" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -8915,13 +8891,13 @@
         <v>60</v>
       </c>
       <c r="T14" s="20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U14" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="165" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:21" ht="165" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -8947,7 +8923,7 @@
       </c>
       <c r="I15" s="9"/>
       <c r="J15" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K15" s="5" t="s">
         <v>85</v>
@@ -8971,13 +8947,13 @@
         <v>90</v>
       </c>
       <c r="T15" s="20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U15" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="54" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:21" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -9001,14 +8977,14 @@
       </c>
       <c r="I16" s="9"/>
       <c r="J16" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K16" s="5" t="s">
         <v>93</v>
       </c>
       <c r="L16" s="9"/>
       <c r="M16" s="9" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="N16" s="9"/>
       <c r="O16" s="9"/>
@@ -9023,10 +8999,10 @@
         <v>96</v>
       </c>
       <c r="T16" s="20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U16" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="17" spans="1:21" ht="80.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9053,7 +9029,7 @@
       </c>
       <c r="I17" s="9"/>
       <c r="J17" s="9" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="K17" s="5" t="s">
         <v>99</v>
@@ -9062,13 +9038,13 @@
         <v>100</v>
       </c>
       <c r="M17" s="9" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="P17" s="9" t="s">
         <v>102</v>
@@ -9079,13 +9055,13 @@
         <v>103</v>
       </c>
       <c r="T17" s="20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U17" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="18" spans="1:21" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:21" ht="83.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -9129,13 +9105,13 @@
         <v>110</v>
       </c>
       <c r="T18" s="20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="U18" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -9165,13 +9141,13 @@
       <c r="R19" s="5"/>
       <c r="S19" s="14"/>
       <c r="T19" s="20" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U19" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="62" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" ht="62" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -9195,18 +9171,18 @@
       </c>
       <c r="I20" s="9"/>
       <c r="J20" s="9" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="K20" s="5" t="s">
         <v>114</v>
       </c>
       <c r="L20" s="9"/>
       <c r="M20" s="9" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="N20" s="9"/>
       <c r="O20" s="9" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="P20" s="9" t="s">
         <v>75</v>
@@ -9217,13 +9193,13 @@
         <v>116</v>
       </c>
       <c r="T20" s="20" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U20" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -9255,10 +9231,10 @@
         <v>60</v>
       </c>
       <c r="T21" s="20" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U21" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="22" spans="1:21" ht="270" x14ac:dyDescent="0.2">
@@ -9295,10 +9271,10 @@
         <v>108</v>
       </c>
       <c r="N22" s="9" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="O22" s="9" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="P22" s="9" t="s">
         <v>20</v>
@@ -9311,13 +9287,13 @@
         <v>122</v>
       </c>
       <c r="T22" s="20" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U22" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="75" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:21" ht="45" x14ac:dyDescent="0.2">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -9341,14 +9317,14 @@
       </c>
       <c r="I23" s="9"/>
       <c r="J23" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K23" s="5" t="s">
         <v>125</v>
       </c>
       <c r="L23" s="9"/>
       <c r="M23" s="9" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="N23" s="9"/>
       <c r="O23" s="9"/>
@@ -9363,13 +9339,13 @@
         <v>128</v>
       </c>
       <c r="T23" s="20" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U23" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:21" ht="30" x14ac:dyDescent="0.2">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -9391,14 +9367,14 @@
       <c r="H24" s="5"/>
       <c r="I24" s="9"/>
       <c r="J24" s="9" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="K24" s="5" t="s">
         <v>131</v>
       </c>
       <c r="L24" s="9"/>
       <c r="M24" s="9" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="N24" s="9"/>
       <c r="O24" s="9"/>
@@ -9411,10 +9387,10 @@
       <c r="R24" s="5"/>
       <c r="S24" s="14"/>
       <c r="T24" s="20" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U24" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="25" spans="1:21" ht="135" x14ac:dyDescent="0.2">
@@ -9441,20 +9417,20 @@
         <v>137</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="K25" s="5"/>
       <c r="L25" s="9" t="s">
         <v>135</v>
       </c>
       <c r="M25" s="9" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="P25" s="9" t="s">
         <v>20</v>
@@ -9469,10 +9445,10 @@
         <v>140</v>
       </c>
       <c r="T25" s="20" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U25" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="26" spans="1:21" ht="135" x14ac:dyDescent="0.2">
@@ -9499,20 +9475,20 @@
         <v>143</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="K26" s="5"/>
       <c r="L26" s="9" t="s">
         <v>135</v>
       </c>
       <c r="M26" s="9" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="N26" s="9" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="P26" s="9" t="s">
         <v>144</v>
@@ -9527,10 +9503,10 @@
         <v>140</v>
       </c>
       <c r="T26" s="20" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U26" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="27" spans="1:21" ht="135" x14ac:dyDescent="0.2">
@@ -9544,7 +9520,7 @@
       <c r="C27" s="8"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="5" t="s">
@@ -9553,20 +9529,20 @@
       <c r="H27" s="5"/>
       <c r="I27" s="9"/>
       <c r="J27" s="9" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="K27" s="5"/>
       <c r="L27" s="9" t="s">
         <v>135</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="P27" s="9"/>
       <c r="Q27" s="9" t="s">
@@ -9577,13 +9553,13 @@
         <v>140</v>
       </c>
       <c r="T27" s="20" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="U27" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="28" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -9615,13 +9591,13 @@
         <v>60</v>
       </c>
       <c r="T28" s="20" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="U28" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="29" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -9653,13 +9629,13 @@
         <v>60</v>
       </c>
       <c r="T29" s="20" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="U29" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="30" spans="1:21" ht="80" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:21" ht="50" x14ac:dyDescent="0.2">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -9681,14 +9657,14 @@
       <c r="H30" s="5"/>
       <c r="I30" s="9"/>
       <c r="J30" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>152</v>
       </c>
       <c r="L30" s="9"/>
       <c r="M30" s="9" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="N30" s="9"/>
       <c r="O30" s="9"/>
@@ -9703,13 +9679,13 @@
         <v>154</v>
       </c>
       <c r="T30" s="20" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="U30" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -9741,13 +9717,13 @@
         <v>60</v>
       </c>
       <c r="T31" s="20" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="U31" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="119.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:21" ht="119.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -9765,7 +9741,7 @@
         <v>157</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>159</v>
@@ -9773,7 +9749,7 @@
       <c r="H32" s="5"/>
       <c r="I32" s="9"/>
       <c r="J32" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K32" s="5" t="s">
         <v>158</v>
@@ -9799,13 +9775,13 @@
         <v>162</v>
       </c>
       <c r="T32" s="20" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="U32" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="33" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -9837,13 +9813,13 @@
         <v>60</v>
       </c>
       <c r="T33" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U33" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="34" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:21" ht="40" x14ac:dyDescent="0.2">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -9871,7 +9847,7 @@
       </c>
       <c r="I34" s="11"/>
       <c r="J34" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K34" s="5" t="s">
         <v>166</v>
@@ -9895,13 +9871,13 @@
         <v>172</v>
       </c>
       <c r="T34" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U34" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="35" spans="1:21" ht="100" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:21" ht="90" x14ac:dyDescent="0.2">
       <c r="A35" s="4">
         <v>34</v>
       </c>
@@ -9925,7 +9901,7 @@
       </c>
       <c r="I35" s="9"/>
       <c r="J35" s="9" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="K35" s="5" t="s">
         <v>175</v>
@@ -9936,7 +9912,7 @@
       </c>
       <c r="N35" s="9"/>
       <c r="O35" s="9" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="P35" s="8">
         <v>7</v>
@@ -9947,13 +9923,13 @@
         <v>116</v>
       </c>
       <c r="T35" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U35" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="36" spans="1:21" ht="83.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:21" ht="83.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -9971,7 +9947,7 @@
         <v>179</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="G36" s="5"/>
       <c r="H36" s="5" t="s">
@@ -9999,13 +9975,13 @@
         <v>184</v>
       </c>
       <c r="T36" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U36" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="37" spans="1:21" ht="81.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:21" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4">
         <v>36</v>
       </c>
@@ -10049,13 +10025,13 @@
         <v>191</v>
       </c>
       <c r="T37" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U37" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="38" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A38" s="4">
         <v>37</v>
       </c>
@@ -10087,10 +10063,10 @@
         <v>60</v>
       </c>
       <c r="T38" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U38" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="39" spans="1:21" ht="180" x14ac:dyDescent="0.2">
@@ -10108,7 +10084,7 @@
         <v>193</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
@@ -10121,13 +10097,13 @@
       <c r="K39" s="5"/>
       <c r="L39" s="9"/>
       <c r="M39" s="9" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="P39" s="9" t="s">
         <v>12</v>
@@ -10140,13 +10116,13 @@
         <v>197</v>
       </c>
       <c r="T39" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U39" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="40" spans="1:21" ht="388.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:21" ht="388.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4">
         <v>39</v>
       </c>
@@ -10172,18 +10148,18 @@
       </c>
       <c r="I40" s="9"/>
       <c r="J40" s="9" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="K40" s="5" t="s">
         <v>200</v>
       </c>
       <c r="L40" s="9"/>
       <c r="M40" s="9" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="N40" s="9"/>
       <c r="O40" s="9" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="P40" s="9" t="s">
         <v>20</v>
@@ -10196,13 +10172,13 @@
         <v>204</v>
       </c>
       <c r="T40" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U40" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="41" spans="1:21" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4">
         <v>40</v>
       </c>
@@ -10234,13 +10210,13 @@
         <v>60</v>
       </c>
       <c r="T41" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U41" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="42" spans="1:21" ht="119.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:21" ht="119.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4">
         <v>41</v>
       </c>
@@ -10264,7 +10240,7 @@
       <c r="H42" s="5"/>
       <c r="I42" s="9"/>
       <c r="J42" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K42" s="5" t="s">
         <v>208</v>
@@ -10290,13 +10266,13 @@
         <v>211</v>
       </c>
       <c r="T42" s="20" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U42" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="43" spans="1:21" ht="70" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:21" ht="61" x14ac:dyDescent="0.2">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -10340,13 +10316,13 @@
         <v>219</v>
       </c>
       <c r="T43" s="9" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="U43" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="44" spans="1:21" ht="56" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:21" ht="56" x14ac:dyDescent="0.2">
       <c r="A44" s="4">
         <v>43</v>
       </c>
@@ -10370,7 +10346,7 @@
         <v>223</v>
       </c>
       <c r="J44" s="9" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="K44" s="5"/>
       <c r="L44" s="9"/>
@@ -10390,13 +10366,13 @@
         <v>226</v>
       </c>
       <c r="T44" s="9" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="U44" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="45" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -10428,13 +10404,13 @@
         <v>60</v>
       </c>
       <c r="T45" s="9" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="U45" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="46" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:21" ht="30" x14ac:dyDescent="0.2">
       <c r="A46" s="4">
         <v>45</v>
       </c>
@@ -10470,13 +10446,13 @@
       <c r="R46" s="5"/>
       <c r="S46" s="14"/>
       <c r="T46" s="9" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="U46" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="47" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:21" ht="40" x14ac:dyDescent="0.2">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -10500,7 +10476,7 @@
       <c r="H47" s="5"/>
       <c r="I47" s="9"/>
       <c r="J47" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K47" s="5" t="s">
         <v>234</v>
@@ -10524,13 +10500,13 @@
         <v>237</v>
       </c>
       <c r="T47" s="9" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="U47" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="48" spans="1:21" ht="40" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:21" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -10552,7 +10528,7 @@
       <c r="H48" s="5"/>
       <c r="I48" s="9"/>
       <c r="J48" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K48" s="5" t="s">
         <v>240</v>
@@ -10576,13 +10552,13 @@
         <v>243</v>
       </c>
       <c r="T48" s="9" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="U48" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="119.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:21" ht="119.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -10606,7 +10582,7 @@
       <c r="H49" s="5"/>
       <c r="I49" s="9"/>
       <c r="J49" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K49" s="5" t="s">
         <v>246</v>
@@ -10632,13 +10608,13 @@
         <v>248</v>
       </c>
       <c r="T49" s="9" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="U49" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -10670,13 +10646,13 @@
         <v>60</v>
       </c>
       <c r="T50" s="9" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="U50" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:21" ht="40" x14ac:dyDescent="0.2">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -10704,7 +10680,7 @@
       </c>
       <c r="I51" s="9"/>
       <c r="J51" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K51" s="5" t="s">
         <v>252</v>
@@ -10728,13 +10704,13 @@
         <v>257</v>
       </c>
       <c r="T51" s="9" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="U51" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:21" ht="30" x14ac:dyDescent="0.2">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -10759,7 +10735,7 @@
       <c r="K52" s="5"/>
       <c r="L52" s="9"/>
       <c r="M52" s="9" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="N52" s="9"/>
       <c r="O52" s="9"/>
@@ -10774,13 +10750,13 @@
         <v>261</v>
       </c>
       <c r="T52" s="9" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="U52" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="53" spans="1:21" ht="119.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:21" ht="119.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4">
         <v>52</v>
       </c>
@@ -10804,7 +10780,7 @@
       <c r="H53" s="5"/>
       <c r="I53" s="9"/>
       <c r="J53" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K53" s="5" t="s">
         <v>264</v>
@@ -10828,13 +10804,13 @@
         <v>268</v>
       </c>
       <c r="T53" s="9" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="U53" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A54" s="4">
         <v>53</v>
       </c>
@@ -10866,13 +10842,13 @@
         <v>60</v>
       </c>
       <c r="T54" s="9" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="U54" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="55" spans="1:21" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4">
         <v>54</v>
       </c>
@@ -10904,13 +10880,13 @@
         <v>60</v>
       </c>
       <c r="T55" s="9" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="U55" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="120" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:21" ht="90" x14ac:dyDescent="0.2">
       <c r="A56" s="4">
         <v>55</v>
       </c>
@@ -10932,14 +10908,14 @@
       <c r="H56" s="5"/>
       <c r="I56" s="9"/>
       <c r="J56" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K56" s="5" t="s">
         <v>273</v>
       </c>
       <c r="L56" s="9"/>
       <c r="M56" s="9" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="N56" s="9"/>
       <c r="O56" s="9"/>
@@ -10954,10 +10930,10 @@
         <v>275</v>
       </c>
       <c r="T56" s="9" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="U56" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="57" spans="1:21" ht="167.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -10984,16 +10960,16 @@
       </c>
       <c r="I57" s="9"/>
       <c r="J57" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K57" s="5" t="s">
         <v>278</v>
       </c>
       <c r="L57" s="17" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="M57" s="9" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="N57" s="9" t="s">
         <v>280</v>
@@ -11012,13 +10988,13 @@
         <v>282</v>
       </c>
       <c r="T57" s="9" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="U57" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="84.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:21" ht="84.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4">
         <v>57</v>
       </c>
@@ -11044,7 +11020,7 @@
       </c>
       <c r="I58" s="9"/>
       <c r="J58" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K58" s="5" t="s">
         <v>285</v>
@@ -11068,13 +11044,13 @@
         <v>290</v>
       </c>
       <c r="T58" s="9" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="U58" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="59" spans="1:21" ht="169.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:21" ht="169.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="4">
         <v>58</v>
       </c>
@@ -11104,14 +11080,14 @@
         <v>297</v>
       </c>
       <c r="J59" s="13" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K59" s="5" t="s">
         <v>293</v>
       </c>
       <c r="L59" s="9"/>
       <c r="M59" s="9" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="N59" s="9"/>
       <c r="O59" s="9"/>
@@ -11122,19 +11098,19 @@
         <v>298</v>
       </c>
       <c r="R59" s="5" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="S59" s="14" t="s">
         <v>299</v>
       </c>
       <c r="T59" s="9" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="U59" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="99" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:21" ht="99" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="4">
         <v>59</v>
       </c>
@@ -11148,7 +11124,7 @@
         <v>300</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="G60" s="5"/>
       <c r="H60" s="6" t="s">
@@ -11163,7 +11139,7 @@
         <v>301</v>
       </c>
       <c r="M60" s="9" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="N60" s="9"/>
       <c r="O60" s="9"/>
@@ -11176,13 +11152,13 @@
         <v>304</v>
       </c>
       <c r="T60" s="9" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="U60" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="61" spans="1:21" ht="87" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:21" ht="87" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="4">
         <v>60</v>
       </c>
@@ -11211,7 +11187,7 @@
         <v>106</v>
       </c>
       <c r="M61" s="9" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="N61" s="9"/>
       <c r="O61" s="9"/>
@@ -11226,13 +11202,13 @@
         <v>309</v>
       </c>
       <c r="T61" s="9" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="U61" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="62" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A62" s="4">
         <v>61</v>
       </c>
@@ -11264,13 +11240,13 @@
         <v>60</v>
       </c>
       <c r="T62" s="9" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="U62" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="63" spans="1:21" ht="75" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:21" ht="75" x14ac:dyDescent="0.2">
       <c r="A63" s="4">
         <v>62</v>
       </c>
@@ -11304,13 +11280,13 @@
         <v>313</v>
       </c>
       <c r="T63" s="9" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="U63" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="64" spans="1:21" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="4">
         <v>63</v>
       </c>
@@ -11342,13 +11318,13 @@
         <v>60</v>
       </c>
       <c r="T64" s="9" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="U64" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="65" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:21" ht="40" x14ac:dyDescent="0.2">
       <c r="A65" s="4">
         <v>64</v>
       </c>
@@ -11372,7 +11348,7 @@
       <c r="H65" s="5"/>
       <c r="I65" s="9"/>
       <c r="J65" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K65" s="5" t="s">
         <v>317</v>
@@ -11394,10 +11370,10 @@
         <v>320</v>
       </c>
       <c r="T65" s="9" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="U65" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="66" spans="1:21" ht="183" x14ac:dyDescent="0.2">
@@ -11414,7 +11390,7 @@
         <v>321</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G66" s="5"/>
       <c r="H66" s="5" t="s">
@@ -11429,13 +11405,13 @@
         <v>17</v>
       </c>
       <c r="M66" s="9" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="N66" s="9" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="O66" s="9" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="P66" s="9" t="s">
         <v>88</v>
@@ -11450,10 +11426,10 @@
         <v>326</v>
       </c>
       <c r="T66" s="9" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="U66" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="67" spans="1:21" ht="212" x14ac:dyDescent="0.2">
@@ -11470,7 +11446,7 @@
         <v>327</v>
       </c>
       <c r="F67" s="9" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="G67" s="5"/>
       <c r="H67" s="5" t="s">
@@ -11485,13 +11461,13 @@
         <v>328</v>
       </c>
       <c r="M67" s="9" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="P67" s="9" t="s">
         <v>75</v>
@@ -11503,16 +11479,16 @@
         <v>325</v>
       </c>
       <c r="S67" s="16" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="T67" s="9" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="U67" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="68" spans="1:21" ht="210" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:21" ht="210" x14ac:dyDescent="0.2">
       <c r="A68" s="4">
         <v>67</v>
       </c>
@@ -11550,13 +11526,13 @@
         <v>335</v>
       </c>
       <c r="T68" s="9" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="U68" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="69" spans="1:21" ht="370" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:21" ht="370" x14ac:dyDescent="0.2">
       <c r="A69" s="4">
         <v>68</v>
       </c>
@@ -11584,7 +11560,7 @@
       </c>
       <c r="I69" s="11"/>
       <c r="J69" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K69" s="5" t="s">
         <v>338</v>
@@ -11610,13 +11586,13 @@
         <v>343</v>
       </c>
       <c r="T69" s="9" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="U69" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="70" spans="1:21" ht="190" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:21" ht="130" x14ac:dyDescent="0.2">
       <c r="A70" s="4">
         <v>69</v>
       </c>
@@ -11638,17 +11614,17 @@
       <c r="H70" s="5"/>
       <c r="I70" s="9"/>
       <c r="J70" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K70" s="5" t="s">
         <v>346</v>
       </c>
       <c r="L70" s="9"/>
       <c r="M70" s="9" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N70" s="9" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="O70" s="9"/>
       <c r="P70" s="9" t="s">
@@ -11662,13 +11638,13 @@
         <v>348</v>
       </c>
       <c r="T70" s="9" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="U70" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="71" spans="1:21" ht="114" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:21" ht="114" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="4">
         <v>70</v>
       </c>
@@ -11686,7 +11662,7 @@
         <v>350</v>
       </c>
       <c r="F71" s="9" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="G71" s="5"/>
       <c r="H71" s="5" t="s">
@@ -11701,7 +11677,7 @@
         <v>351</v>
       </c>
       <c r="M71" s="9" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="N71" s="9"/>
       <c r="O71" s="9"/>
@@ -11718,13 +11694,13 @@
         <v>355</v>
       </c>
       <c r="T71" s="9" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="U71" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="72" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:21" ht="40" x14ac:dyDescent="0.2">
       <c r="A72" s="4">
         <v>71</v>
       </c>
@@ -11746,14 +11722,14 @@
       <c r="H72" s="5"/>
       <c r="I72" s="9"/>
       <c r="J72" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K72" s="5" t="s">
         <v>358</v>
       </c>
       <c r="L72" s="9"/>
       <c r="M72" s="9" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="N72" s="9"/>
       <c r="O72" s="9"/>
@@ -11768,10 +11744,10 @@
         <v>360</v>
       </c>
       <c r="T72" s="9" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="U72" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="73" spans="1:21" ht="76.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -11798,7 +11774,7 @@
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="9" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="K73" s="5" t="s">
         <v>363</v>
@@ -11807,13 +11783,13 @@
         <v>364</v>
       </c>
       <c r="M73" s="9" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="P73" s="9" t="s">
         <v>75</v>
@@ -11824,13 +11800,13 @@
         <v>366</v>
       </c>
       <c r="T73" s="9" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="U73" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="74" spans="1:21" ht="81.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:21" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="4">
         <v>73</v>
       </c>
@@ -11876,13 +11852,13 @@
         <v>372</v>
       </c>
       <c r="T74" s="9" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="U74" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="75" spans="1:21" ht="85.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:21" ht="85.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="4">
         <v>74</v>
       </c>
@@ -11924,13 +11900,13 @@
         <v>376</v>
       </c>
       <c r="T75" s="9" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="U75" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="76" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:21" ht="40" x14ac:dyDescent="0.2">
       <c r="A76" s="4">
         <v>75</v>
       </c>
@@ -11952,14 +11928,14 @@
       <c r="H76" s="5"/>
       <c r="I76" s="9"/>
       <c r="J76" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K76" s="5" t="s">
         <v>379</v>
       </c>
       <c r="L76" s="9"/>
       <c r="M76" s="9" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="N76" s="9"/>
       <c r="O76" s="9"/>
@@ -11967,7 +11943,7 @@
         <v>12</v>
       </c>
       <c r="Q76" s="9" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="R76" s="5" t="s">
         <v>380</v>
@@ -11976,13 +11952,13 @@
         <v>381</v>
       </c>
       <c r="T76" s="9" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="U76" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="77" spans="1:21" ht="20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A77" s="4">
         <v>76</v>
       </c>
@@ -12014,13 +11990,13 @@
         <v>60</v>
       </c>
       <c r="T77" s="9" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="U77" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="78" spans="1:21" ht="90" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:21" ht="60" x14ac:dyDescent="0.2">
       <c r="A78" s="4">
         <v>77</v>
       </c>
@@ -12056,13 +12032,13 @@
         <v>385</v>
       </c>
       <c r="T78" s="9" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="U78" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="79" spans="1:21" ht="225" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:21" ht="225" x14ac:dyDescent="0.2">
       <c r="A79" s="4">
         <v>78</v>
       </c>
@@ -12085,7 +12061,7 @@
         <v>387</v>
       </c>
       <c r="M79" s="24" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="N79" s="13"/>
       <c r="O79" s="13"/>
@@ -12098,13 +12074,13 @@
         <v>388</v>
       </c>
       <c r="T79" s="9" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="U79" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="80" spans="1:21" ht="48.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:21" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="4">
         <v>79</v>
       </c>
@@ -12146,13 +12122,13 @@
         <v>394</v>
       </c>
       <c r="T80" s="9" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="U80" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="81" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:21" ht="20" x14ac:dyDescent="0.2">
       <c r="A81" s="4">
         <v>80</v>
       </c>
@@ -12184,13 +12160,13 @@
         <v>60</v>
       </c>
       <c r="T81" s="9" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="U81" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="82" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:21" ht="40" x14ac:dyDescent="0.2">
       <c r="A82" s="4">
         <v>81</v>
       </c>
@@ -12212,14 +12188,14 @@
       <c r="H82" s="5"/>
       <c r="I82" s="9"/>
       <c r="J82" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K82" s="5" t="s">
         <v>398</v>
       </c>
       <c r="L82" s="9"/>
       <c r="M82" s="9" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="N82" s="9"/>
       <c r="O82" s="9"/>
@@ -12234,13 +12210,13 @@
         <v>400</v>
       </c>
       <c r="T82" s="9" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="U82" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="83" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:21" ht="40" x14ac:dyDescent="0.2">
       <c r="A83" s="4">
         <v>82</v>
       </c>
@@ -12262,14 +12238,14 @@
       <c r="H83" s="5"/>
       <c r="I83" s="9"/>
       <c r="J83" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K83" s="5" t="s">
         <v>403</v>
       </c>
       <c r="L83" s="9"/>
       <c r="M83" s="9" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="N83" s="9"/>
       <c r="O83" s="9"/>
@@ -12284,13 +12260,13 @@
         <v>405</v>
       </c>
       <c r="T83" s="9" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="U83" s="20" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="84" spans="1:21" ht="49" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:21" ht="49" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="4">
         <v>83</v>
       </c>
@@ -12324,13 +12300,13 @@
       <c r="R84" s="5"/>
       <c r="S84" s="14"/>
       <c r="T84" s="9" t="s">
+        <v>502</v>
+      </c>
+      <c r="U84" s="20" t="s">
         <v>503</v>
       </c>
-      <c r="U84" s="20" t="s">
-        <v>504</v>
-      </c>
     </row>
-    <row r="85" spans="1:21" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:21" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="4">
         <v>84</v>
       </c>
@@ -12348,7 +12324,7 @@
         <v>409</v>
       </c>
       <c r="F85" s="9" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="G85" s="5"/>
       <c r="H85" s="7" t="s">
@@ -12356,7 +12332,7 @@
       </c>
       <c r="I85" s="13"/>
       <c r="J85" s="13" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K85" s="5" t="s">
         <v>410</v>
@@ -12377,16 +12353,16 @@
         <v>413</v>
       </c>
       <c r="S85" s="16" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="T85" s="9" t="s">
+        <v>502</v>
+      </c>
+      <c r="U85" s="20" t="s">
         <v>503</v>
       </c>
-      <c r="U85" s="20" t="s">
-        <v>504</v>
-      </c>
     </row>
-    <row r="86" spans="1:21" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:21" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="4">
         <v>85</v>
       </c>
@@ -12404,7 +12380,7 @@
         <v>415</v>
       </c>
       <c r="F86" s="9" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="G86" s="5"/>
       <c r="H86" s="5" t="s">
@@ -12412,7 +12388,7 @@
       </c>
       <c r="I86" s="9"/>
       <c r="J86" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K86" s="5" t="s">
         <v>416</v>
@@ -12434,13 +12410,13 @@
         <v>419</v>
       </c>
       <c r="T86" s="9" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="U86" s="20" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
-    <row r="87" spans="1:21" ht="209" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:21" ht="209" x14ac:dyDescent="0.2">
       <c r="A87" s="4">
         <v>86</v>
       </c>
@@ -12468,7 +12444,7 @@
         <v>425</v>
       </c>
       <c r="J87" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K87" s="5" t="s">
         <v>422</v>
@@ -12477,7 +12453,7 @@
         <v>17</v>
       </c>
       <c r="M87" s="9" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="N87" s="9"/>
       <c r="O87" s="9"/>
@@ -12492,13 +12468,13 @@
         <v>427</v>
       </c>
       <c r="T87" s="9" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="U87" s="20" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
-    <row r="88" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:21" ht="45" x14ac:dyDescent="0.2">
       <c r="A88" s="4">
         <v>87</v>
       </c>
@@ -12522,7 +12498,7 @@
       </c>
       <c r="I88" s="9"/>
       <c r="J88" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K88" s="5" t="s">
         <v>430</v>
@@ -12533,7 +12509,7 @@
       </c>
       <c r="N88" s="9"/>
       <c r="O88" s="9" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="P88" s="9" t="s">
         <v>12</v>
@@ -12546,13 +12522,13 @@
         <v>434</v>
       </c>
       <c r="T88" s="9" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="U88" s="20" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
-    <row r="89" spans="1:21" ht="245" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:21" ht="245" x14ac:dyDescent="0.2">
       <c r="A89" s="4">
         <v>88</v>
       </c>
@@ -12567,10 +12543,10 @@
         <v>435</v>
       </c>
       <c r="E89" s="9" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="F89" s="9" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G89" s="5"/>
       <c r="H89" s="5" t="s">
@@ -12578,14 +12554,14 @@
       </c>
       <c r="I89" s="9"/>
       <c r="J89" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K89" s="5" t="s">
         <v>436</v>
       </c>
       <c r="L89" s="9"/>
       <c r="M89" s="9" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="N89" s="9"/>
       <c r="O89" s="9"/>
@@ -12602,13 +12578,13 @@
         <v>439</v>
       </c>
       <c r="T89" s="9" t="s">
+        <v>505</v>
+      </c>
+      <c r="U89" s="20" t="s">
         <v>506</v>
       </c>
-      <c r="U89" s="20" t="s">
-        <v>507</v>
-      </c>
     </row>
-    <row r="90" spans="1:21" ht="55" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:21" ht="55" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="4">
         <v>89</v>
       </c>
@@ -12619,7 +12595,7 @@
       <c r="C90" s="8"/>
       <c r="D90" s="9"/>
       <c r="E90" s="9" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F90" s="9"/>
       <c r="G90" s="5"/>
@@ -12640,13 +12616,13 @@
         <v>440</v>
       </c>
       <c r="T90" s="9" t="s">
+        <v>505</v>
+      </c>
+      <c r="U90" s="20" t="s">
         <v>506</v>
       </c>
-      <c r="U90" s="20" t="s">
-        <v>507</v>
-      </c>
     </row>
-    <row r="91" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:21" ht="60" x14ac:dyDescent="0.2">
       <c r="A91" s="4">
         <v>90</v>
       </c>
@@ -12678,13 +12654,13 @@
       <c r="R91" s="5"/>
       <c r="S91" s="14"/>
       <c r="T91" s="9" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="U91" s="20" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
-    <row r="92" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:21" ht="60" x14ac:dyDescent="0.2">
       <c r="A92" s="4">
         <v>91</v>
       </c>
@@ -12718,13 +12694,13 @@
       <c r="R92" s="5"/>
       <c r="S92" s="14"/>
       <c r="T92" s="9" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="U92" s="20" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
-    <row r="93" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:21" ht="60" x14ac:dyDescent="0.2">
       <c r="A93" s="4">
         <v>92</v>
       </c>
@@ -12748,7 +12724,7 @@
       <c r="H93" s="5"/>
       <c r="I93" s="9"/>
       <c r="J93" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K93" s="5" t="s">
         <v>447</v>
@@ -12768,13 +12744,13 @@
       <c r="R93" s="5"/>
       <c r="S93" s="14"/>
       <c r="T93" s="9" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="U93" s="20" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
-    <row r="94" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:21" ht="30" x14ac:dyDescent="0.2">
       <c r="A94" s="4">
         <v>93</v>
       </c>
@@ -12794,7 +12770,7 @@
       <c r="H94" s="5"/>
       <c r="I94" s="9"/>
       <c r="J94" s="9" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K94" s="5" t="s">
         <v>451</v>
@@ -12814,13 +12790,13 @@
       <c r="R94" s="5"/>
       <c r="S94" s="14"/>
       <c r="T94" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U94" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="95" spans="1:21" ht="86.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:21" ht="86.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="4">
         <v>94</v>
       </c>
@@ -12847,7 +12823,7 @@
         <v>106</v>
       </c>
       <c r="M95" s="9" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="N95" s="9"/>
       <c r="O95" s="9"/>
@@ -12862,13 +12838,13 @@
         <v>455</v>
       </c>
       <c r="T95" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U95" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="96" spans="1:21" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:21" ht="60" x14ac:dyDescent="0.2">
       <c r="A96" s="4">
         <v>95</v>
       </c>
@@ -12879,7 +12855,7 @@
       <c r="C96" s="8"/>
       <c r="D96" s="9"/>
       <c r="E96" s="9" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F96" s="9"/>
       <c r="G96" s="5"/>
@@ -12889,7 +12865,7 @@
       <c r="K96" s="5"/>
       <c r="L96" s="9"/>
       <c r="M96" s="9" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="N96" s="9"/>
       <c r="O96" s="9"/>
@@ -12902,13 +12878,13 @@
       <c r="R96" s="5"/>
       <c r="S96" s="14"/>
       <c r="T96" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U96" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="97" spans="1:21" ht="105" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:21" ht="105" x14ac:dyDescent="0.2">
       <c r="A97" s="4">
         <v>96</v>
       </c>
@@ -12919,14 +12895,14 @@
       <c r="C97" s="8"/>
       <c r="D97" s="9"/>
       <c r="E97" s="9" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F97" s="9"/>
       <c r="G97" s="5"/>
       <c r="H97" s="5"/>
       <c r="I97" s="9"/>
       <c r="J97" s="9" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="K97" s="5"/>
       <c r="L97" s="9"/>
@@ -12938,13 +12914,13 @@
       <c r="R97" s="5"/>
       <c r="S97" s="14"/>
       <c r="T97" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U97" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="98" spans="1:21" ht="105" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:21" ht="105" x14ac:dyDescent="0.2">
       <c r="A98" s="4">
         <v>97</v>
       </c>
@@ -12955,14 +12931,14 @@
       <c r="C98" s="8"/>
       <c r="D98" s="9"/>
       <c r="E98" s="9" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F98" s="9"/>
       <c r="G98" s="5"/>
       <c r="H98" s="5"/>
       <c r="I98" s="9"/>
       <c r="J98" s="9" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="K98" s="5"/>
       <c r="L98" s="9"/>
@@ -12974,13 +12950,13 @@
       <c r="R98" s="5"/>
       <c r="S98" s="14"/>
       <c r="T98" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U98" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="99" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:21" ht="30" x14ac:dyDescent="0.2">
       <c r="A99" s="4">
         <v>98</v>
       </c>
@@ -12998,14 +12974,14 @@
       <c r="H99" s="5"/>
       <c r="I99" s="9"/>
       <c r="J99" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K99" s="5" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L99" s="9"/>
       <c r="M99" s="9" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="N99" s="9"/>
       <c r="O99" s="9"/>
@@ -13014,13 +12990,13 @@
       <c r="R99" s="5"/>
       <c r="S99" s="14"/>
       <c r="T99" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U99" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="100" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:21" ht="30" x14ac:dyDescent="0.2">
       <c r="A100" s="4">
         <v>99</v>
       </c>
@@ -13038,14 +13014,14 @@
       <c r="H100" s="5"/>
       <c r="I100" s="9"/>
       <c r="J100" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K100" s="5" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="L100" s="9"/>
       <c r="M100" s="9" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="N100" s="9"/>
       <c r="O100" s="9"/>
@@ -13054,13 +13030,13 @@
       <c r="R100" s="5"/>
       <c r="S100" s="14"/>
       <c r="T100" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U100" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="101" spans="1:21" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:21" ht="30" x14ac:dyDescent="0.2">
       <c r="A101" s="4">
         <v>100</v>
       </c>
@@ -13078,14 +13054,14 @@
       <c r="H101" s="5"/>
       <c r="I101" s="9"/>
       <c r="J101" s="9" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K101" s="5" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="L101" s="9"/>
       <c r="M101" s="9" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="N101" s="9"/>
       <c r="O101" s="9"/>
@@ -13094,13 +13070,13 @@
       <c r="R101" s="5"/>
       <c r="S101" s="14"/>
       <c r="T101" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U101" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="102" spans="1:21" ht="75" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:21" ht="45" x14ac:dyDescent="0.2">
       <c r="A102" s="4">
         <v>101</v>
       </c>
@@ -13111,22 +13087,22 @@
       <c r="C102" s="8"/>
       <c r="D102" s="9"/>
       <c r="E102" s="9" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="F102" s="9"/>
       <c r="G102" s="5"/>
       <c r="H102" s="5"/>
       <c r="I102" s="9"/>
       <c r="J102" s="9" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K102" s="5"/>
       <c r="L102" s="9"/>
       <c r="M102" s="9" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="N102" s="9" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="O102" s="9"/>
       <c r="P102" s="9"/>
@@ -13134,13 +13110,13 @@
       <c r="R102" s="5"/>
       <c r="S102" s="14"/>
       <c r="T102" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U102" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="103" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A103" s="4">
         <v>102</v>
       </c>
@@ -13150,7 +13126,7 @@
       <c r="C103" s="8"/>
       <c r="D103" s="9"/>
       <c r="E103" s="22" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="F103" s="9"/>
       <c r="G103" s="5"/>
@@ -13160,7 +13136,7 @@
       <c r="K103" s="5"/>
       <c r="L103" s="9"/>
       <c r="M103" s="9" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="N103" s="9"/>
       <c r="O103" s="9"/>
@@ -13169,13 +13145,13 @@
       <c r="R103" s="5"/>
       <c r="S103" s="14"/>
       <c r="T103" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U103" s="20" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="104" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:21" ht="15" x14ac:dyDescent="0.2">
       <c r="A104" s="4">
         <v>103</v>
       </c>
@@ -13195,7 +13171,7 @@
       <c r="K104" s="5"/>
       <c r="L104" s="9"/>
       <c r="M104" s="9" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="N104" s="9"/>
       <c r="O104" s="9"/>
@@ -13204,7 +13180,7 @@
       <c r="R104" s="5"/>
       <c r="S104" s="14"/>
       <c r="T104" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="U104" s="20" t="s">
         <v>450</v>

</xml_diff>